<commit_message>
feat: Synchronize refined 11 acupoint reports, FMA 5.1.0/US integration, master DB sync v3.0, and WORKLOG
</commit_message>
<xml_diff>
--- a/01_경혈별_해부생리_분석보고서/BL_족태양방광경/BL02_찬죽/BL02_찬죽_해부생리_분석데이터.xlsx
+++ b/01_경혈별_해부생리_분석보고서/BL_족태양방광경/BL02_찬죽/BL02_찬죽_해부생리_분석데이터.xlsx
@@ -18,6 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LayerA_papers" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="외부검색로그" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개정이력" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FMA_해부실체" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -502,7 +503,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -894,6 +894,101 @@
         <v>30</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-23T21:43:19</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>pubmed</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>200</v>
+      </c>
+      <c r="D6" t="n">
+        <v>16</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>("BL2" OR "Cuanzhu" OR "攒竹") AND (acupuncture OR electroacupuncture) AND (nerve OR reflex OR autonomic OR mechanism OR anatomy) | ("BL2" OR "Cuanzhu" OR "攒竹") AND ("Zhongguo Zhen Jiu"[Journal] OR "Zhen Ci Yan Jiu"[Journal])</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-23T21:43:19</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>openalex</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>200</v>
+      </c>
+      <c r="D7" t="n">
+        <v>23</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>doi_starts_with:10.13703,title_and_abstract.search:"Cuanzhu" OR "BL2" | doi_starts_with:10.13702,title_and_abstract.search:"Cuanzhu" OR "BL2" | has_doi:true,title_and_abstract.search:"Cuanzhu" OR "BL2" AND (acupuncture OR electroacupuncture)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-23T21:43:19</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>crossref</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>200</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Cuanzhu acupuncture nerve reflex</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-23T21:43:19</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>40</v>
+      </c>
+      <c r="E9" t="n">
+        <v>37</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>merged_into_existing=27 batch_dups=10 sources={'pubmed': 'ok', 'openalex': 'ok', 'crossref': 'ok'}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -905,7 +1000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1131,6 +1226,692 @@
       <c r="D10" t="inlineStr">
         <is>
           <t>final_BL02.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>FMA_해부실체 시트 신설 (2026-10-23)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>FMA 5.1.0 실체 ID·지배신경·줄기·분절·교재 비교 추가, 횡단면 모식도·FMA 경로도 추가. ARI·B-Check 불변</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>fma_query.py profile BL02; 보고서 4·6·8절·부록 A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>교재 용어</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>FMA_ID</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>FMA_label</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>대응 수준</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>출처 교재</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>지배신경(FMA nerve_supply)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>상위 줄기(FMA)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>척수 분절(FMA segmental_supply)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>근육</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>눈썹주름근 (corrugator supercilii)</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>46794</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Corrugator supercilii</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>공통교재·김재효</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>FMA:53379 Nerve to corrugator supercilii</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Temporal branch of facial nerve → Facial nerve</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>FMA 미기재</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>근육</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>눈썹내림근 (depressor supercilii)</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>46798</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Depressor supercilii</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>김재효</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>FMA:82674 Nerve to depressor supercilii</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Temporal branch of facial nerve → Facial nerve</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>FMA 미기재</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>근육</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>뒤통수이마근의 이마힘살 (frontal belly of the occipitofrontalis); 이마힘살 (frontal belly)</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>46757</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Frontalis</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>공통교재·김재효</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>FMA 미기재</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>FMA nerve_supply 미기재 → B1-01(얼굴신경 관자가지)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>근육</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>눈둘레근 (orbicularis oculi)</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>46779</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Orbicularis oculi</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>공통교재·김재효</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>FMA:53314 Branch of zygomatic branch of facial nerve to orbicularis oculi; FMA:53377 Branch of temporal branch of facial nerve to orbicularis oculi</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Zygomatic branch of facial nerve → Facial nerve</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>FMA 미기재</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>신경</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>얼굴신경 (facial nerve)</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>50868</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Facial nerve</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>공통교재</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>FMA 미기재</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>신경</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>이마신경 (frontal nerve)</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>52638</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Frontal nerve</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>공통교재</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>FMA:52621 Ophthalmic nerve → FMA:50866 Trigeminal nerve</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>FMA 미기재</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>신경</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>눈확위신경 (supraorbital nerve)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>52655</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Supra-orbital nerve</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>김재효</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>FMA:52638 Frontal nerve → FMA:52621 Ophthalmic nerve → FMA:50866 Trigeminal nerve</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>FMA 미기재</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>단면 밖(바깥쪽)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>신경</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>도르래위신경 (supratrochlear nerve)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>52642</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Supratrochlear nerve</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>김재효</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>FMA:52638 Frontal nerve → FMA:52621 Ophthalmic nerve → FMA:50866 Trigeminal nerve</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>FMA 미기재</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>신경</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>얼굴신경의 관자가지 (temporal branch of the facial nerve)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>53291</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Temporal branch of facial nerve</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>김재효</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>FMA:50868 Facial nerve</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>FMA 미기재</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>혈관</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>눈확위동ㆍ정맥 (supraorbial artery and vein)</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>49973</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Supra-orbital artery</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>김재효</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>FMA:49868 Ophthalmic artery → FMA:3947 Internal carotid artery → FMA:3939 Common carotid artery</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>FMA 미기재</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>额切迹 바깥 眶上切迹 통과 — BL02 단면 밖</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>혈관</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>눈확위동ㆍ정맥 (supraorbial artery and vein)</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>50904</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Supra-orbital vein</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>김재효</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>FMA:50893 Angular vein → FMA:50874 Facial vein → FMA:4724 Internal jugular vein → FMA:4723 Brachiocephalic vein</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>FMA 미기재</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>단면 밖(바깥쪽)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>혈관</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>도르래위동ㆍ정맥 (supratrochlear artery and vein)</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>50025</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Supratrochlear artery</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>공통교재·김재효</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>FMA:49868 Ophthalmic artery → FMA:3947 Internal carotid artery → FMA:3939 Common carotid artery</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>FMA 미기재</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>혈관</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>도르래위동ㆍ정맥 (supratrochlear artery and vein)</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>50898</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Supratrochlear vein</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>공통교재·김재효</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>FMA:50893 Angular vein → FMA:50874 Facial vein → FMA:4724 Internal jugular vein → FMA:4723 Brachiocephalic vein</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>FMA 미기재</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>눈구석정맥-위눈정맥 교통은 FMA 미기재(B1-01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>분절 합집합</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>FMA 기재 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>교재 비교</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>공통 5 · 공통교재 단독 2 · 김재효 단독 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>출처</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>FMA 5.1.0 로컬 색인, fma_query.py profile BL02 (2026-10-23). B1 보조(등록부 미등재)</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1952,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -1431,7 +2211,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -1726,7 +2505,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -1927,7 +2705,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -2123,7 +2900,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(reports): apply Tri-Target and 经络通鉴 collation to 12 Tier 3 reports
- All 12 category-1 reports (ko/en md + html, analysis xlsx): add
  《中国针灸经络通鉴》 rows, align 《证治通鉴》 with the Korean translation,
  re-assess targets with pairwise Δ tables under the 10mm threshold
- ST36: new Target 2 (TA–EDL septum), dual-scored 56.25 ± 1.25 (C·H);
  Target 1≡3 (77.5 ± 0, B) confirmed superior
- PC09: S_orig ④ 50 → 75 from 经络通鉴 collation, ARI-Core 70.0 ± 1.2 (B,
  weight-sensitive)
- LU06: Sawada Kongzui excluded from Targets under the exclusion rule
- WORKLOG: chronology rows and report index updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_경혈별_해부생리_분석보고서/BL_족태양방광경/BL02_찬죽/BL02_찬죽_해부생리_분석데이터.xlsx
+++ b/01_경혈별_해부생리_분석보고서/BL_족태양방광경/BL02_찬죽/BL02_찬죽_해부생리_분석데이터.xlsx
@@ -9,16 +9,18 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="종합분석요약" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="문헌고증_DB" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자입심도_고금비교" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="층위별_해부신경구조" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고대언어_현대매핑" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="구판_ARI_정량평가표" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ARI_v3.0" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B-Check" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LayerA_papers" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="외부검색로그" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개정이력" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FMA_해부실체" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="문헌스크리닝_4대원전" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자입심도_고금비교" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="층위별_해부신경구조" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고대언어_현대매핑" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="구판_ARI_정량평가표" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ARI_v3.0" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="분기추론_TriTarget" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B-Check" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LayerA_papers" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="외부검색로그" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개정이력" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FMA_해부실체" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -105,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -116,6 +118,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -720,6 +728,694 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>채점자 A</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>채점자 B</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>최종</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Layer B 참조 ID</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>papers.id</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>근거 요지(A)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>근거 요지(B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>① 심도 말초신경·혈관</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>B1-01, B1-03, B1-05, B2-09</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2대 국내 교재(경혈 특이)와 규범 해부서가 额切迹의 도르래위 신경혈관속·눈썹주름근·눈둘레근 실체를 일치 기술. 영상 실측 논문은 없음.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2대 교재(B2-09)와 通考 해부 기술이 额切迹의 도르래위 신경·동정맥, 눈썹주름근·눈둘레근을 명시적으로 일치시킴. 영상 실측은 없음.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>② 분절(V1 영역) 정합</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>B1-01, B1-02</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>척수 분절 대신 삼차신경 V1 영역 정합: 도르래위신경(V1 이마신경 분지) 피부영역 ↔ 각막·결막·눈물샘 감각(V1)으로 주치(目痛·流淚·眉稜骨痛)와 동일 신경 영역. B3 등록부는 척수 분절 중심이라 뇌신경은 B1로 판단.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>자극 부위 감각신경(도르래위신경, V1)과 표적 기관(안구·결막·눈물샘 감각, V1 영역)이 같은 삼차신경 안신경 분포 안에 있음. 두면부라 척수 분절 대신 삼차신경 영역 정합으로 판정함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>③ 구심 섬유·수용체</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>B3-06</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>기니피그 각막·삼차신경절 P2X3/PKC(동물, 복합 혈위). 섬유형 직접 규명 없음 → 동물 한정 1.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>기니피그 건성안 모델의 삼차신경절 P2X3 변화(1998)만 있음. 동물·다혈 배합이고, BL2 구심 섬유형을 직접 측정한 연구는 없음.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>④ 중추 중계</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>B3-05, B3-07, B3-11</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>삼차신경 척수핵·상타액핵 경로는 등록부 범위 밖 유추. 삼차신경절 수준 동물 자료만.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>삼차신경 척수핵 중계는 유추에 그침. 중추 경로를 측정한 Layer A 논문은 없음.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>⑤ 원심·효과 방향</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>B3-14</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1981, 1997, 1999</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>눈물분비 증가(VIP/AQP5)·안구표면 항염증(α7nAChR/NF-κB)이 流淚·目赤腫痛 주치 방향과 일치하나 동물·복합혈위, B3-14는 침 연구 아닌 범위 밖 틀 → 1.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>동물 모델에서 눈물 분비 증가·안표면 항염증(α7nAChR 콜린성)이 확인되어 目赤肿痛·目疾 주치 방향과 대체로 맞음. 다만 고전 주치 '流泪/迎风冷泪'(유루 과다)와 건성안 모델(분비 촉진)의 효과 방향은 직접 대응하지 않아 유추 수준임.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>⑥ 인체 전환</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>B4-04, B4-05</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1979, 1994, 2000</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>인체 RCT(건성안)·안륜근 기능 연구가 있으나 복합 혈위·가침 대조 불명확, 신경영상·자율지표 없음. 혈위 특이성 미입증 → 1.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>인체 RCT·임상연구가 있으나 다혈 배합·점안제 병용이라 BL2 혈위 특이성을 분리하지 못함(B4-05 반증 측면 검토 필요).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>8</v>
+      </c>
+      <c r="C8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>판정: 부합</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>동물 한정 표지 없음(⑥=1), 가설 제한 없음</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Layer A 전부 복합 혈위 — BL2 단독 연구 0편</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>papers.id</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>연도</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>저널</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>제목</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>PMID</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>DOI</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>설계·BL2 관련성</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1979</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Zhongguo Zhen Jiu</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Effect of acupuncture on dry eye and tear inflammatory factors</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>36484191</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>10.13703/j.0255-2930.20220318-0001</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>인체 임상(건성안), 복합 혈위</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1981</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Zhen Ci Yan Jiu</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Acupuncture mitigates ocular surface inflammatory response via α7nAChR/NF-κB p65 signaling in dry eye guinea pigs</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>36453674</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>10.13702/j.1000-0607.20220015</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>동물(기니피그), 복합 혈위</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1994</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Zhongguo Zhen Jiu</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Penetrating needling of three eye acupoints combined with sodium hyaluronate eye drops for dry eye: an RCT</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>40369920</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>10.13703/j.0255-2930.20240521-0002</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>인체 RCT, 3혈 투자+점안제</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1997</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Zhen Ci Yan Jiu</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Acupuncture promotes tear secretion by up-regulating VIP/cAMP/PKA/AQP5 signaling in guinea pigs</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>37879953</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>10.13702/j.1000-0607.20230061</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>동물(기니피그), 복합 혈위</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1998</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Zhen Ci Yan Jiu</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Effect of electroacupuncture on ocular surface sensory neuralgia and P2X3/PKC in cornea and trigeminal ganglion</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>35616412</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>10.13702/j.1000-0607.20210607</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>동물(기니피그), 복합 혈위</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1999</v>
+      </c>
+      <c r="B7" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Zhen Ci Yan Jiu</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Effect of acupuncture on expression of TGF-β1 in lacrimal gland of rabbits with dry eye</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>32959555</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>10.13702/j.1000-0607.190977</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>동물(토끼), 복합 혈위</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B8" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Zhen Ci Yan Jiu</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Influence on orbicularis oculi muscle in facial neuritis treated with penetrating needling</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>32959557</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>10.13702/j.1000-0607.190894</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>인체 비RCT, BL2→EX-HN4 투자+BL62</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2001</v>
+      </c>
+      <c r="B9" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Zhen Ci Yan Jiu</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Acupuncture of intraorbital and extraorbital acupoints reduces apoptosis of retinal ganglion</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>31056882</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>10.13702/j.1000-0607.180440</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>동물(토끼 NAION), 복합 혈위</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B10" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PubMed(pack 표기)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Acupuncture alleviates form-deprivation myopia by promoting dopamine secretion and suppressing ferroptosis</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>42779258</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>10.14670/hh-25-141</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>동물(근시), 복합 혈위, 채점자 B만 계수</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B11" t="n">
+        <v>2003</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>J Acupunct Tuina Sci</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Treatment of 55 cases of acute lumbar sprain by puncturing acupoint Cuanzhu (BL 2)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>10.1007/bf02845431</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>참고: BL2 단독, 요추 염좌 증례군 — 채점 미사용</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -994,13 +1690,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1251,12 +1947,34 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Framework 2.7.7 (2026-10-25)</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>3대 원전; 단일 Target T1(편차 15mm 미만); S_orig④ 通考 교감; 证治通鉴 PDF 기준 포인터</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>4대 원전(经络通鉴 24·27·12편 — 문헌스크리닝_4대원전 시트); Tri-Target 재점검 Target 1≡2≡3(쌍별 Δ ≤ 10mm 추정, 분기 기준 Δ&gt;10mm) — 분기추론_TriTarget 시트; 眉本(太素 手少阳 = 丝竹空) 혼용 차단 기록, ③ 75 유지; ④ 通考·经络通鉴 교감 재점검 불변; 证治通鉴 18·20·23·06편 포인터+한글번역; ARI·SI 점수 불변</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>프레임워크 2.7.7–2.7.8; data/classics/中国针灸经络通鉴/ 12·24·27편; data/classics/中国针灸证治通鉴/ 06·18·20·23편(+한글번역)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2185,6 +2903,547 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>원전</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>편·인용 문헌</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>파일 (내부 포인터)</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>행</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>원문 발췌</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>판정·비고</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>보고서 위치</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>中国针灸经络通鉴</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>24편 《素问·气府论》 足太阳脉气所发</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>data/classics/中国针灸经络通鉴/中国针灸经络通鉴_24_第叁编_第七篇_足太阳经脉、经别、络脉和经筋.md</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>L333</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>足太阳脉气所发者七十八穴：两眉头各一…</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>위치 = 眉头(明堂과 일치)</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>1절 15b</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>中国针灸经络通鉴</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>24편 《太素·气府》 杨上善 注</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>data/classics/中国针灸经络通鉴/中国针灸经络通鉴_24_第叁编_第七篇_足太阳经脉、经别、络脉和经筋.md</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>L337</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>［足太阳脉气所发者七十三穴：两眉头各一］攒竹二穴也</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>杨注 = 攒竹</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>1절 15b</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>中国针灸经络通鉴</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>24편 《素问·气府论》 王冰 注</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>data/classics/中国针灸经络通鉴/中国针灸经络通鉴_24_第叁编_第七篇_足太阳经脉、经别、络脉和经筋.md</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>L341</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>［两眉头各一。］谓攒竹穴也，所刺灸分壮与气穴同</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>王注 = 攒竹</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>1절 15b</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>中国针灸经络通鉴</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>24편 《灵枢·口问》 / 《太素·十二邪》</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>data/classics/中国针灸经络通鉴/中国针灸经络通鉴_24_第叁编_第七篇_足太阳经脉、经别、络脉和经筋.md</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>L2115, L2119</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>嚏者，补足太阳，眉本。 / 嚏，补足太阳，眉本。</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>眉本 = 부위명(足太阳 문맥)</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>1절 15c, 3절</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>中国针灸经络通鉴</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>27편 《素问·气府论》 手少阳 / 《太素·气府》 杨注 / 王冰 注</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>data/classics/中国针灸经络通鉴/中国针灸经络通鉴_27_第叁编_第十篇_手少阳经脉、经别、络脉和经筋.md</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>L287, L291, L300</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>眉后各一 / ［眉本各一，］丝竹空，左右二穴 / ［眉后各一，］谓丝竹空二穴也</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>本/后 이문, 太素 문맥 眉本 = 丝竹空(TE23) → 혼용 위험, 按 없음(미해결)</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>1절 15d, 3절, S_orig④ 재점검</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>中国针灸经络通鉴</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>24편 足太阳 경맥 순행 주석(《十四经发挥》·张介宾·《经络汇编》 등)</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>data/classics/中国针灸经络通鉴/中国针灸经络通鉴_24_第叁编_第七篇_足太阳经脉、经别、络脉和经筋.md</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>L128, L178, L189, L218, L228</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>足太阳起目内眦睛明穴，上额，循攒竹…</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>후대 주석이 순행에 攒竹 삽입; 위치 변화 없음</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>1절 15e</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>中国针灸经络通鉴</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>24편 《医学纲目·目疾门》</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>data/classics/中国针灸经络通鉴/中国针灸经络通鉴_24_第叁编_第七篇_足太阳经脉、经别、络脉和经筋.md</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>L2424</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>乃刺其鼻中攒竹穴，与烦前五穴，大出血，目立明</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>사혈 증례; "烦前" 판본 대조 못 함</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>1절 15f</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>中国针灸经络通鉴</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>12편 《灵枢·卫气》 手阳明 标</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>data/classics/中国针灸经络通鉴/中国针灸经络通鉴_12_第贰编_第四篇_经络的标本、气街与四海.md</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>L91</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>手阳明之本，在肘骨中…标在颜下合钳上也</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>"在颜下" 유일 출현 — 찬죽 무관(구판 가공 인용 검증)</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>1절 각주</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>中国针灸经络通鉴</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>전수 검색</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>data/classics/中国针灸经络通鉴/*.md</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>乌列/烏列/大空 0건, 禁用针灸 0건</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>3·5절 문구 갱신 근거</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>3·5절</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>中国针灸证治通鉴</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>18편 二十八.呕吐·反胃 — 呃逆</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>data/classics/中国针灸证治通鉴/中国针灸证治通鉴_18_第叁编_内科病症_二十五劳瘵至三十消渴.md</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>L1168 (한글번역 L1857)</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>取穴：攒竹。指压。（浙江中医杂志，1980…；广西中医药，1990…）</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>구 포인터 "PDF 241–320쪽 2254행" 대체</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>1절 15, 9절</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>中国针灸证治通鉴</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>20편 四十.腰痛 附：现代针灸文献选录</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>data/classics/中国针灸证治通鉴/中国针灸证治通鉴_20_第叁编_内科病症_三十九霍乱至四十二遗精.md</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>L661 (한글번역 L1120)</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>取穴：攒竹。（中国针灸，1982，2（3）：47）</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>구 포인터 "PDF 321–400쪽 14행" 대체</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>1절 15, 9절</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>中国针灸证治通鉴</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>23편 目病 — 《针灸玉龙经·玉龙歌》</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>data/classics/中国针灸证治通鉴/中国针灸证治通鉴_23_第叁编_五官病证_目病_耳病.md</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>L186 (한글번역 L291–293)</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>眉目疼痛不能当，攒竹沿皮刺不妨。</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>구 포인터 "PDF 401–480쪽 184행" 대체</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>1절 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>中国针灸证治通鉴</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>06편 足太阳膀胱经(上) 二)攒竹</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>data/classics/中国针灸证治通鉴/中国针灸证治通鉴_06_第壹编_第七篇_足太阳膀胱经(上).md</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>L30–58 (한글번역 L36–58)</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>《明堂经》 主风头痛…目䀮䀮不明，恶风寒。 / 《灵枢》 主噫，嚏。</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>신규 수록</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>1절 15a</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2475,7 +3734,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2674,7 +3933,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2870,7 +4129,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3056,7 +4315,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3108,7 +4367,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Target 1≡2≡3 (구 T1)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3134,7 +4393,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Target 1≡2≡3 (구 T1)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3160,7 +4419,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Target 1≡2≡3 (구 T1)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3186,7 +4445,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Target 1≡2≡3 (구 T1)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3212,12 +4471,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Target 1≡2≡3 (구 T1)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>S_orig ④ 通考 교감</t>
+          <t>S_orig ④ 通考·经络通鉴 교감</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -3231,14 +4490,14 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>员在 形误, 脉动应手 错入, 聚英 承泣 주치, 额切迹</t>
+          <t>员在 形误, 脉动应手 错入, 聚英 承泣 주치, 额切迹 | 2026-10-25 经络通鉴 재점검(24편 L333–341·2115·2119, 27편 L287·291·300): 정위 문구 교감 없음, 眉本/眉后 이문 미판정 → 단계 이동 없음, 불변</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Target 1≡2≡3 (구 T1)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3264,7 +4523,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Target 1≡2≡3 (구 T1)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3290,7 +4549,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Target 1≡2≡3 (구 T1)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3315,6 +4574,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -3407,7 +4667,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>단일 Target, 해당 없음</t>
+          <t>Tri-Target 재점검: Target 1≡2≡3 단일 Target(쌍별 Δ ≤ 10mm 추정), 해당 없음 — 분기추론_TriTarget 시트</t>
         </is>
       </c>
     </row>
@@ -3432,309 +4692,6 @@
       <c r="B20" t="inlineStr">
         <is>
           <t>S_safety 75점 불일치(A 0 / B 75): 두 채점자 모두 《穴位通鉴》·《针灸腧穴通考》(上)_561-640.md 【操作】9항에 수록된 《医学入门》 卷一 '禁用针灸' 기록을 확인함. 정본 4.2 SI 0단계('금침 문헌 존재')를 문언대로 적용하여 B를 0으로 조정 → ⚠ 안전주의. 단, 자침깊이 DB의 다수 문헌은 1~3푼(2.3~6.9mm)으로 금침 기록은 단일 후대 문헌임을 본문에 병기. conflicts 기록은 직접 상충이 아니므로 B-Check '가설' 미적용.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>항목</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>채점자 A</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>채점자 B</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>최종</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Layer B 참조 ID</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>papers.id</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>근거 요지(A)</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>근거 요지(B)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>① 심도 말초신경·혈관</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>B1-01, B1-03, B1-05, B2-09</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2대 국내 교재(경혈 특이)와 규범 해부서가 额切迹의 도르래위 신경혈관속·눈썹주름근·눈둘레근 실체를 일치 기술. 영상 실측 논문은 없음.</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2대 교재(B2-09)와 通考 해부 기술이 额切迹의 도르래위 신경·동정맥, 눈썹주름근·눈둘레근을 명시적으로 일치시킴. 영상 실측은 없음.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>② 분절(V1 영역) 정합</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>B1-01, B1-02</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>척수 분절 대신 삼차신경 V1 영역 정합: 도르래위신경(V1 이마신경 분지) 피부영역 ↔ 각막·결막·눈물샘 감각(V1)으로 주치(目痛·流淚·眉稜骨痛)와 동일 신경 영역. B3 등록부는 척수 분절 중심이라 뇌신경은 B1로 판단.</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>자극 부위 감각신경(도르래위신경, V1)과 표적 기관(안구·결막·눈물샘 감각, V1 영역)이 같은 삼차신경 안신경 분포 안에 있음. 두면부라 척수 분절 대신 삼차신경 영역 정합으로 판정함.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>③ 구심 섬유·수용체</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>B3-06</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>1998</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>기니피그 각막·삼차신경절 P2X3/PKC(동물, 복합 혈위). 섬유형 직접 규명 없음 → 동물 한정 1.</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>기니피그 건성안 모델의 삼차신경절 P2X3 변화(1998)만 있음. 동물·다혈 배합이고, BL2 구심 섬유형을 직접 측정한 연구는 없음.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>④ 중추 중계</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>B3-05, B3-07, B3-11</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>1998</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>삼차신경 척수핵·상타액핵 경로는 등록부 범위 밖 유추. 삼차신경절 수준 동물 자료만.</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>삼차신경 척수핵 중계는 유추에 그침. 중추 경로를 측정한 Layer A 논문은 없음.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>⑤ 원심·효과 방향</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>B3-14</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>1981, 1997, 1999</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>눈물분비 증가(VIP/AQP5)·안구표면 항염증(α7nAChR/NF-κB)이 流淚·目赤腫痛 주치 방향과 일치하나 동물·복합혈위, B3-14는 침 연구 아닌 범위 밖 틀 → 1.</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>동물 모델에서 눈물 분비 증가·안표면 항염증(α7nAChR 콜린성)이 확인되어 目赤肿痛·目疾 주치 방향과 대체로 맞음. 다만 고전 주치 '流泪/迎风冷泪'(유루 과다)와 건성안 모델(분비 촉진)의 효과 방향은 직접 대응하지 않아 유추 수준임.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>⑥ 인체 전환</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>B4-04, B4-05</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>1979, 1994, 2000</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>인체 RCT(건성안)·안륜근 기능 연구가 있으나 복합 혈위·가침 대조 불명확, 신경영상·자율지표 없음. 혈위 특이성 미입증 → 1.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>인체 RCT·임상연구가 있으나 다혈 배합·점안제 병용이라 BL2 혈위 특이성을 분리하지 못함(B4-05 반증 측면 검토 필요).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>합계</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>8</v>
-      </c>
-      <c r="C8" t="n">
-        <v>8</v>
-      </c>
-      <c r="D8" t="n">
-        <v>8</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>판정: 부합</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>동물 한정 표지 없음(⑥=1), 가설 제한 없음</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Layer A 전부 복합 혈위 — BL2 단독 연구 0편</t>
         </is>
       </c>
     </row>
@@ -3749,377 +4706,263 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>papers.id</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>연도</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>저널</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>제목</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>PMID</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>DOI</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>설계·BL2 관련성</t>
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>정의</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>원전 근거</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>X·Y 위치(체표)</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>자입 기준점</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>구판 표기 대응</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1979</v>
-      </c>
-      <c r="B2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Zhongguo Zhen Jiu</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Effect of acupuncture on dry eye and tear inflammatory factors</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>36484191</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>10.13703/j.0255-2930.20220318-0001</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>인체 임상(건성안), 복합 혈위</t>
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Target 1 (고전 문헌 위치)</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>최초 기술 문구 위치</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>《明堂》(甲乙 卷三) 在眉头陷者中; 素问·气府论 两眉头各一(杨注·王注 = 攒竹, 经络通鉴 24편 L333–341)</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>눈썹머리 오목</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>v2.7 단일 Target T1 → Target 1≡2≡3</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>1981</v>
-      </c>
-      <c r="B3" t="n">
-        <v>2022</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Zhen Ci Yan Jiu</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Acupuncture mitigates ocular surface inflammatory response via α7nAChR/NF-κB p65 signaling in dry eye guinea pigs</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>36453674</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>10.13702/j.1000-0607.20220015</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>동물(기니피그), 복합 혈위</t>
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Target 2 (촉진 실체화 위치)</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>陷者中이 가리키는 해부 공간</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>通考 部位 "眉头凹陷中，额切迹处", 相关解剖学基础; 窦氏 两眉头内尖陷中</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>이마뼈 额切迹(FMA:57409)</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>간극 표현 없음 → 형식상 미표시; 촉진 실체 = 骨性 오목 额切迹(덮는 근육 FMA:46794·46779, 통과 FMA:52642·50025·50898)</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>신규(2026-10-25), Target 1·3과 병합</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>1994</v>
-      </c>
-      <c r="B4" t="n">
-        <v>2025</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Zhongguo Zhen Jiu</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Penetrating needling of three eye acupoints combined with sodium hyaluronate eye drops for dry eye: an RCT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>40369920</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>10.13703/j.0255-2930.20240521-0002</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>인체 RCT, 3혈 투자+점안제</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>1997</v>
-      </c>
-      <c r="B5" t="n">
-        <v>2023</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Zhen Ci Yan Jiu</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Acupuncture promotes tear secretion by up-regulating VIP/cAMP/PKA/AQP5 signaling in guinea pigs</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>37879953</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>10.13702/j.1000-0607.20230061</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>동물(기니피그), 복합 혈위</t>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Target 3 (WHO 표준 위치)</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>현대 표준 정위</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>WHO 2008 (B1-05) In the depression at the medial end of the eyebrow</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>눈썹 내측단 오목</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Target 1≡2≡3</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>1998</v>
-      </c>
-      <c r="B6" t="n">
-        <v>2022</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Zhen Ci Yan Jiu</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Effect of electroacupuncture on ocular surface sensory neuralgia and P2X3/PKC in cornea and trigeminal ganglion</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>35616412</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>10.13702/j.1000-0607.20210607</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>동물(기니피그), 복합 혈위</t>
-        </is>
-      </c>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>쌍</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Δ (추정)</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>추정 근거</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>판정 (Δ &gt; 10mm 분기)</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>15mm→10mm 기준 변경 영향</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>1999</v>
-      </c>
-      <c r="B7" t="n">
-        <v>2020</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Zhen Ci Yan Jiu</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Effect of acupuncture on expression of TGF-β1 in lacrimal gland of rabbits with dry eye</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>32959555</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>10.13702/j.1000-0607.190977</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>동물(토끼), 복합 혈위</t>
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Target 1–Target 2</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>≤ 10mm (추정)</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>T1 문구 자체가 陷者中; 通考가 额切迹으로 동정; 古代文献无分歧</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>병합</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>변화 없음</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>2000</v>
-      </c>
-      <c r="B8" t="n">
-        <v>2020</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Zhen Ci Yan Jiu</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Influence on orbicularis oculi muscle in facial neuritis treated with penetrating needling</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>32959557</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>10.13702/j.1000-0607.190894</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>인체 비RCT, BL2→EX-HN4 투자+BL62</t>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Target 1–Target 3</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>≤ 10mm (추정)</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>WHO 문구 = 眉头陷者中의 직역</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>병합</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>변화 없음</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>2001</v>
-      </c>
-      <c r="B9" t="n">
-        <v>2019</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Zhen Ci Yan Jiu</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Acupuncture of intraorbital and extraorbital acupoints reduces apoptosis of retinal ganglion</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>31056882</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>10.13702/j.1000-0607.180440</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>동물(토끼 NAION), 복합 혈위</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>2003</v>
-      </c>
-      <c r="B10" t="n">
-        <v>2026</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>PubMed(pack 표기)</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Acupuncture alleviates form-deprivation myopia by promoting dopamine secretion and suppressing ferroptosis</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>42779258</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>10.14670/hh-25-141</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>동물(근시), 복합 혈위, 채점자 B만 계수</t>
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Target 2–Target 3</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>≤ 10mm (추정)</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>같은 골성 오목 기준; 눈썹머리 개인차 있으나 골성 기준이라 편차 작음; BL2 실측 없음</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>병합</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>변화 없음</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>2008</v>
-      </c>
-      <c r="B11" t="n">
-        <v>2003</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>J Acupunct Tuina Sci</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Treatment of 55 cases of acute lumbar sprain by puncturing acupoint Cuanzhu (BL 2)</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>10.1007/bf02845431</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>참고: BL2 단독, 요추 염좌 증례군 — 채점 미사용</t>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>판정</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Target 1≡2≡3 단일 Target — Rank 7 Tri-Target ΔARI 판정 대상 없음. 점수는 v2.7 이중 채점(A·B) 승계, 단일 채점(예비) Target 없음.</t>
         </is>
       </c>
     </row>

</xml_diff>